<commit_message>
Kimyasal Ekim dosyası: MT657 TURQUOISE BLUE 14 Ekim çıkış 135 -> 0,135 düzeltildi
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01J6foNXTwf1dGzDjULYpfrk
</commit_message>
<xml_diff>
--- a/kimyasal/2026-10_Baski_Kimyasal_Tuketim.xlsx
+++ b/kimyasal/2026-10_Baski_Kimyasal_Tuketim.xlsx
@@ -16,7 +16,7 @@
     <sheet name="Instructions التعليمات" sheetId="1" r:id="rId1"/>
     <sheet name="Monthly Consumption" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191029" fullCalcOnLoad="1"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -16114,14 +16114,14 @@
       </c>
       <c r="CK32" s="9"/>
       <c r="CL32" s="9">
-        <v>135</v>
+        <v>0.135</v>
       </c>
       <c r="CM32" s="9">
         <v>0</v>
       </c>
       <c r="CN32" s="8">
         <f t="shared" si="38"/>
-        <v>135</v>
+        <v>0.135</v>
       </c>
       <c r="CO32" s="8">
         <f t="shared" si="39"/>

</xml_diff>